<commit_message>
tyarchive extension, scrape wmo .py, 蒙古实况高低温
</commit_message>
<xml_diff>
--- a/气象/For_Python_站点信息和记录.xlsx
+++ b/气象/For_Python_站点信息和记录.xlsx
@@ -817,8 +817,8 @@
     <col width="18.59765625" customWidth="1" style="8" min="25" max="25"/>
     <col width="12.59765625" customWidth="1" style="5" min="26" max="30"/>
     <col width="12.59765625" customWidth="1" style="8" min="31" max="32"/>
-    <col width="12.59765625" customWidth="1" style="5" min="33" max="422"/>
-    <col width="12.59765625" customWidth="1" style="5" min="423" max="16384"/>
+    <col width="12.59765625" customWidth="1" style="5" min="33" max="433"/>
+    <col width="12.59765625" customWidth="1" style="5" min="434" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customFormat="1" customHeight="1" s="11">
@@ -1041,13 +1041,13 @@
         </is>
       </c>
       <c r="O2" s="32" t="n">
-        <v>2.8</v>
+        <v>6.3</v>
       </c>
       <c r="P2" s="32" t="n">
-        <v>27.3</v>
+        <v>24.2</v>
       </c>
       <c r="Q2" s="32" t="n">
-        <v>15.64</v>
+        <v>15.07</v>
       </c>
       <c r="R2" s="23" t="inlineStr">
         <is>
@@ -1147,10 +1147,10 @@
         </is>
       </c>
       <c r="O3" s="32" t="n">
-        <v>4.7</v>
+        <v>3.7</v>
       </c>
       <c r="P3" s="32" t="n">
-        <v>25.4</v>
+        <v>22.5</v>
       </c>
       <c r="Q3" s="32" t="n"/>
       <c r="R3" s="23" t="n"/>
@@ -1251,10 +1251,10 @@
         </is>
       </c>
       <c r="O4" s="32" t="n">
-        <v>0.6</v>
+        <v>2.5</v>
       </c>
       <c r="P4" s="32" t="n">
-        <v>24.8</v>
+        <v>23.2</v>
       </c>
       <c r="Q4" s="32" t="n"/>
       <c r="R4" s="23" t="n"/>
@@ -1443,12 +1443,14 @@
         </is>
       </c>
       <c r="O6" s="32" t="n">
-        <v>-4.4</v>
+        <v>-3.5</v>
       </c>
       <c r="P6" s="32" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="Q6" s="32" t="n"/>
+        <v>19</v>
+      </c>
+      <c r="Q6" s="32" t="n">
+        <v>7.46</v>
+      </c>
       <c r="R6" s="23" t="n"/>
       <c r="S6" s="37" t="n"/>
       <c r="T6" s="41" t="inlineStr">
@@ -1543,10 +1545,10 @@
         </is>
       </c>
       <c r="O7" s="32" t="n">
-        <v>-1.5</v>
+        <v>-0.1</v>
       </c>
       <c r="P7" s="32" t="n">
-        <v>20.7</v>
+        <v>17.2</v>
       </c>
       <c r="Q7" s="32" t="n"/>
       <c r="R7" s="23" t="n"/>
@@ -1651,13 +1653,13 @@
       </c>
       <c r="N8" s="2" t="n"/>
       <c r="O8" s="32" t="n">
-        <v>-1.6</v>
+        <v>-4.2</v>
       </c>
       <c r="P8" s="32" t="n">
-        <v>24.8</v>
+        <v>21.5</v>
       </c>
       <c r="Q8" s="32" t="n">
-        <v>11.88</v>
+        <v>9.25</v>
       </c>
       <c r="R8" s="23" t="inlineStr">
         <is>
@@ -1763,13 +1765,13 @@
       </c>
       <c r="N9" s="2" t="n"/>
       <c r="O9" s="32" t="n">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
       <c r="P9" s="32" t="n">
-        <v>26.8</v>
+        <v>23.9</v>
       </c>
       <c r="Q9" s="32" t="n">
-        <v>16.65</v>
+        <v>14.59</v>
       </c>
       <c r="R9" s="23" t="inlineStr">
         <is>
@@ -1883,13 +1885,13 @@
         </is>
       </c>
       <c r="O10" s="32" t="n">
-        <v>-1.8</v>
+        <v>-1</v>
       </c>
       <c r="P10" s="32" t="n">
-        <v>23.3</v>
+        <v>22.3</v>
       </c>
       <c r="Q10" s="32" t="n">
-        <v>11.71</v>
+        <v>12.02</v>
       </c>
       <c r="R10" s="23" t="inlineStr">
         <is>
@@ -1999,13 +2001,13 @@
         </is>
       </c>
       <c r="O11" s="32" t="n">
-        <v>-3.2</v>
+        <v>-3.5</v>
       </c>
       <c r="P11" s="32" t="n">
-        <v>18.9</v>
+        <v>18.6</v>
       </c>
       <c r="Q11" s="32" t="n">
-        <v>9.44</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="R11" s="23" t="inlineStr">
         <is>
@@ -2111,13 +2113,13 @@
       </c>
       <c r="N12" s="2" t="n"/>
       <c r="O12" s="32" t="n">
-        <v>-1.3</v>
+        <v>-1.6</v>
       </c>
       <c r="P12" s="32" t="n">
-        <v>21</v>
+        <v>21.5</v>
       </c>
       <c r="Q12" s="32" t="n">
-        <v>10.75</v>
+        <v>10.56</v>
       </c>
       <c r="R12" s="23" t="inlineStr">
         <is>
@@ -2227,13 +2229,13 @@
         </is>
       </c>
       <c r="O13" s="32" t="n">
-        <v>-2.5</v>
+        <v>-0.3</v>
       </c>
       <c r="P13" s="32" t="n">
-        <v>21</v>
+        <v>18.5</v>
       </c>
       <c r="Q13" s="32" t="n">
-        <v>9.960000000000001</v>
+        <v>8.34</v>
       </c>
       <c r="R13" s="23" t="inlineStr">
         <is>
@@ -2339,13 +2341,13 @@
       </c>
       <c r="N14" s="2" t="n"/>
       <c r="O14" s="32" t="n">
-        <v>2.1</v>
+        <v>-1.5</v>
       </c>
       <c r="P14" s="32" t="n">
-        <v>21.1</v>
+        <v>17.4</v>
       </c>
       <c r="Q14" s="32" t="n">
-        <v>11.31</v>
+        <v>8.15</v>
       </c>
       <c r="R14" s="23" t="inlineStr">
         <is>
@@ -2445,12 +2447,14 @@
       </c>
       <c r="N15" s="2" t="n"/>
       <c r="O15" s="32" t="n">
-        <v>-6.3</v>
+        <v>-9</v>
       </c>
       <c r="P15" s="32" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="Q15" s="32" t="n"/>
+        <v>14.4</v>
+      </c>
+      <c r="Q15" s="32" t="n">
+        <v>3</v>
+      </c>
       <c r="R15" s="23" t="n"/>
       <c r="S15" s="37" t="n"/>
       <c r="T15" s="41" t="inlineStr">
@@ -7673,10 +7677,10 @@
       </c>
       <c r="N73" s="2" t="n"/>
       <c r="O73" s="32" t="n">
-        <v>-6.4</v>
+        <v>-10.3</v>
       </c>
       <c r="P73" s="32" t="n">
-        <v>20.8</v>
+        <v>17.1</v>
       </c>
       <c r="Q73" s="32" t="n"/>
       <c r="R73" s="23" t="n"/>
@@ -8071,13 +8075,13 @@
         </is>
       </c>
       <c r="O77" s="32" t="n">
-        <v>-9.5</v>
+        <v>-0.8</v>
       </c>
       <c r="P77" s="32" t="n">
-        <v>6.9</v>
+        <v>7.8</v>
       </c>
       <c r="Q77" s="32" t="n">
-        <v>-0.49</v>
+        <v>2.43</v>
       </c>
       <c r="R77" s="23" t="inlineStr">
         <is>
@@ -8497,13 +8501,13 @@
         </is>
       </c>
       <c r="O81" s="32" t="n">
-        <v>-6.9</v>
+        <v>-6.8</v>
       </c>
       <c r="P81" s="32" t="n">
-        <v>14.5</v>
+        <v>13.7</v>
       </c>
       <c r="Q81" s="32" t="n">
-        <v>4.49</v>
+        <v>4.56</v>
       </c>
       <c r="R81" s="23" t="inlineStr">
         <is>
@@ -8618,13 +8622,13 @@
         </is>
       </c>
       <c r="O82" s="32" t="n">
-        <v>-6.4</v>
+        <v>-6.8</v>
       </c>
       <c r="P82" s="32" t="n">
-        <v>14.5</v>
+        <v>13.7</v>
       </c>
       <c r="Q82" s="32" t="n">
-        <v>4.34</v>
+        <v>3.79</v>
       </c>
       <c r="R82" s="23" t="inlineStr">
         <is>
@@ -8836,13 +8840,13 @@
         </is>
       </c>
       <c r="O84" s="32" t="n">
-        <v>-3.3</v>
+        <v>-3.6</v>
       </c>
       <c r="P84" s="32" t="n">
-        <v>25.5</v>
+        <v>21</v>
       </c>
       <c r="Q84" s="32" t="n">
-        <v>10.71</v>
+        <v>7.8</v>
       </c>
       <c r="R84" s="23" t="inlineStr">
         <is>
@@ -9054,13 +9058,13 @@
       </c>
       <c r="N86" s="2" t="n"/>
       <c r="O86" s="32" t="n">
-        <v>6.2</v>
+        <v>5.5</v>
       </c>
       <c r="P86" s="32" t="n">
-        <v>28.5</v>
+        <v>21</v>
       </c>
       <c r="Q86" s="32" t="n">
-        <v>18.16</v>
+        <v>13.12</v>
       </c>
       <c r="R86" s="23" t="inlineStr">
         <is>
@@ -9280,13 +9284,13 @@
       </c>
       <c r="N88" s="2" t="n"/>
       <c r="O88" s="32" t="n">
-        <v>1.7</v>
+        <v>0.9</v>
       </c>
       <c r="P88" s="32" t="n">
-        <v>19.7</v>
+        <v>16.8</v>
       </c>
       <c r="Q88" s="32" t="n">
-        <v>11.82</v>
+        <v>10.38</v>
       </c>
       <c r="R88" s="23" t="inlineStr">
         <is>
@@ -9690,13 +9694,13 @@
       </c>
       <c r="N92" s="2" t="n"/>
       <c r="O92" s="32" t="n">
-        <v>0</v>
+        <v>3.1</v>
       </c>
       <c r="P92" s="32" t="n">
-        <v>9.199999999999999</v>
+        <v>11.8</v>
       </c>
       <c r="Q92" s="32" t="n">
-        <v>1.27</v>
+        <v>5.74</v>
       </c>
       <c r="R92" s="23" t="inlineStr">
         <is>
@@ -9802,13 +9806,13 @@
       </c>
       <c r="N93" s="2" t="n"/>
       <c r="O93" s="32" t="n">
-        <v>8.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="P93" s="32" t="n">
-        <v>19.3</v>
+        <v>17.4</v>
       </c>
       <c r="Q93" s="32" t="n">
-        <v>13.47</v>
+        <v>12.81</v>
       </c>
       <c r="R93" s="23" t="inlineStr">
         <is>
@@ -10032,13 +10036,13 @@
       </c>
       <c r="N95" s="2" t="n"/>
       <c r="O95" s="32" t="n">
-        <v>5.3</v>
+        <v>4.5</v>
       </c>
       <c r="P95" s="32" t="n">
-        <v>16.5</v>
+        <v>16.6</v>
       </c>
       <c r="Q95" s="32" t="n">
-        <v>11.71</v>
+        <v>10.7</v>
       </c>
       <c r="R95" s="23" t="inlineStr">
         <is>
@@ -10270,13 +10274,13 @@
       </c>
       <c r="N97" s="2" t="n"/>
       <c r="O97" s="32" t="n">
-        <v>1.7</v>
+        <v>5.2</v>
       </c>
       <c r="P97" s="32" t="n">
-        <v>16.7</v>
+        <v>16.5</v>
       </c>
       <c r="Q97" s="32" t="n">
-        <v>10.52</v>
+        <v>10.99</v>
       </c>
       <c r="R97" s="23" t="inlineStr">
         <is>
@@ -10389,9 +10393,15 @@
         </is>
       </c>
       <c r="N98" s="2" t="n"/>
-      <c r="O98" s="32" t="n"/>
-      <c r="P98" s="32" t="n"/>
-      <c r="Q98" s="32" t="n"/>
+      <c r="O98" s="32" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="P98" s="32" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="Q98" s="32" t="n">
+        <v>10.81</v>
+      </c>
       <c r="R98" s="23" t="inlineStr">
         <is>
           <t>Y</t>
@@ -10826,13 +10836,13 @@
       </c>
       <c r="N102" s="2" t="n"/>
       <c r="O102" s="32" t="n">
-        <v>-6.3</v>
+        <v>-4.9</v>
       </c>
       <c r="P102" s="32" t="n">
-        <v>13.7</v>
+        <v>14.2</v>
       </c>
       <c r="Q102" s="32" t="n">
-        <v>4.85</v>
+        <v>5.03</v>
       </c>
       <c r="R102" s="23" t="inlineStr">
         <is>
@@ -11162,13 +11172,13 @@
         </is>
       </c>
       <c r="O105" s="32" t="n">
-        <v>-8.300000000000001</v>
+        <v>-9.1</v>
       </c>
       <c r="P105" s="32" t="n">
-        <v>12.2</v>
+        <v>13.7</v>
       </c>
       <c r="Q105" s="32" t="n">
-        <v>2.96</v>
+        <v>3.54</v>
       </c>
       <c r="R105" s="23" t="inlineStr">
         <is>
@@ -11996,13 +12006,13 @@
       </c>
       <c r="N113" s="2" t="n"/>
       <c r="O113" s="32" t="n">
-        <v>-8.4</v>
+        <v>-2.8</v>
       </c>
       <c r="P113" s="32" t="n">
-        <v>0.9</v>
+        <v>3.7</v>
       </c>
       <c r="Q113" s="32" t="n">
-        <v>-3.33</v>
+        <v>-1.36</v>
       </c>
       <c r="R113" s="23" t="inlineStr">
         <is>
@@ -12112,13 +12122,13 @@
         </is>
       </c>
       <c r="O114" s="32" t="n">
-        <v>-14.4</v>
+        <v>-3.7</v>
       </c>
       <c r="P114" s="32" t="n">
-        <v>-0.8</v>
+        <v>3.2</v>
       </c>
       <c r="Q114" s="32" t="n">
-        <v>-6.23</v>
+        <v>-1.24</v>
       </c>
       <c r="R114" s="23" t="inlineStr">
         <is>
@@ -12236,13 +12246,13 @@
         </is>
       </c>
       <c r="O115" s="32" t="n">
-        <v>-12.6</v>
+        <v>-5.5</v>
       </c>
       <c r="P115" s="32" t="n">
-        <v>2.6</v>
+        <v>-0.9</v>
       </c>
       <c r="Q115" s="32" t="n">
-        <v>-5.35</v>
+        <v>-3.69</v>
       </c>
       <c r="R115" s="23" t="inlineStr">
         <is>
@@ -12792,13 +12802,13 @@
       </c>
       <c r="N120" s="2" t="n"/>
       <c r="O120" s="32" t="n">
-        <v>18.7</v>
+        <v>18.1</v>
       </c>
       <c r="P120" s="32" t="n">
-        <v>34.8</v>
+        <v>37.3</v>
       </c>
       <c r="Q120" s="32" t="n">
-        <v>27.2</v>
+        <v>28.88</v>
       </c>
       <c r="R120" s="23" t="inlineStr">
         <is>
@@ -12908,13 +12918,13 @@
       </c>
       <c r="N121" s="2" t="n"/>
       <c r="O121" s="32" t="n">
-        <v>15.6</v>
+        <v>15.2</v>
       </c>
       <c r="P121" s="32" t="n">
-        <v>26.6</v>
+        <v>29.3</v>
       </c>
       <c r="Q121" s="32" t="n">
-        <v>21.6</v>
+        <v>22.1</v>
       </c>
       <c r="R121" s="23" t="inlineStr">
         <is>
@@ -13032,13 +13042,13 @@
       </c>
       <c r="N122" s="2" t="n"/>
       <c r="O122" s="32" t="n">
-        <v>-4.3</v>
+        <v>-3.5</v>
       </c>
       <c r="P122" s="32" t="n">
-        <v>18.3</v>
+        <v>18.7</v>
       </c>
       <c r="Q122" s="32" t="n">
-        <v>7.29</v>
+        <v>7.48</v>
       </c>
       <c r="R122" s="23" t="inlineStr">
         <is>
@@ -13254,13 +13264,13 @@
       </c>
       <c r="N124" s="2" t="n"/>
       <c r="O124" s="32" t="n">
-        <v>4.8</v>
+        <v>0.1</v>
       </c>
       <c r="P124" s="32" t="n">
-        <v>18.4</v>
+        <v>18.8</v>
       </c>
       <c r="Q124" s="32" t="n">
-        <v>11.61</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="R124" s="23" t="inlineStr">
         <is>
@@ -13378,13 +13388,13 @@
       </c>
       <c r="N125" s="2" t="n"/>
       <c r="O125" s="32" t="n">
-        <v>6.8</v>
+        <v>14.8</v>
       </c>
       <c r="P125" s="32" t="n">
-        <v>20.9</v>
+        <v>24.5</v>
       </c>
       <c r="Q125" s="32" t="n">
-        <v>14.25</v>
+        <v>19.45</v>
       </c>
       <c r="R125" s="23" t="inlineStr">
         <is>
@@ -13482,13 +13492,13 @@
       </c>
       <c r="N126" s="2" t="n"/>
       <c r="O126" s="32" t="n">
-        <v>9.199999999999999</v>
+        <v>15.4</v>
       </c>
       <c r="P126" s="32" t="n">
-        <v>20.3</v>
+        <v>23.5</v>
       </c>
       <c r="Q126" s="32" t="n">
-        <v>14.4</v>
+        <v>18.56</v>
       </c>
       <c r="R126" s="23" t="inlineStr">
         <is>
@@ -13594,13 +13604,13 @@
       </c>
       <c r="N127" s="2" t="n"/>
       <c r="O127" s="32" t="n">
-        <v>4.8</v>
+        <v>5.3</v>
       </c>
       <c r="P127" s="32" t="n">
-        <v>24.1</v>
+        <v>23.7</v>
       </c>
       <c r="Q127" s="32" t="n">
-        <v>14.58</v>
+        <v>15.35</v>
       </c>
       <c r="R127" s="23" t="inlineStr">
         <is>
@@ -13714,13 +13724,13 @@
       </c>
       <c r="N128" s="2" t="n"/>
       <c r="O128" s="32" t="n">
-        <v>9.1</v>
+        <v>16</v>
       </c>
       <c r="P128" s="32" t="n">
-        <v>25.4</v>
+        <v>24.3</v>
       </c>
       <c r="Q128" s="32" t="n">
-        <v>17.43</v>
+        <v>20.09</v>
       </c>
       <c r="R128" s="23" t="inlineStr">
         <is>
@@ -13826,13 +13836,13 @@
       </c>
       <c r="N129" s="2" t="n"/>
       <c r="O129" s="32" t="n">
-        <v>1.9</v>
+        <v>10.7</v>
       </c>
       <c r="P129" s="32" t="n">
-        <v>24.3</v>
+        <v>21.1</v>
       </c>
       <c r="Q129" s="32" t="n">
-        <v>13.89</v>
+        <v>16.11</v>
       </c>
       <c r="R129" s="23" t="inlineStr">
         <is>
@@ -13946,13 +13956,13 @@
       </c>
       <c r="N130" s="2" t="n"/>
       <c r="O130" s="32" t="n">
-        <v>-1.3</v>
+        <v>5.6</v>
       </c>
       <c r="P130" s="32" t="n">
-        <v>17.5</v>
+        <v>15.8</v>
       </c>
       <c r="Q130" s="32" t="n">
-        <v>7.25</v>
+        <v>9.85</v>
       </c>
       <c r="R130" s="23" t="inlineStr">
         <is>
@@ -14066,13 +14076,13 @@
       </c>
       <c r="N131" s="2" t="n"/>
       <c r="O131" s="32" t="n">
-        <v>11.2</v>
+        <v>13.9</v>
       </c>
       <c r="P131" s="32" t="n">
-        <v>22.4</v>
+        <v>21.4</v>
       </c>
       <c r="Q131" s="32" t="n">
-        <v>14.9</v>
+        <v>17.78</v>
       </c>
       <c r="R131" s="23" t="inlineStr">
         <is>
@@ -14182,13 +14192,13 @@
       </c>
       <c r="N132" s="2" t="n"/>
       <c r="O132" s="32" t="n">
-        <v>11.3</v>
+        <v>19.7</v>
       </c>
       <c r="P132" s="32" t="n">
-        <v>27.6</v>
+        <v>26.7</v>
       </c>
       <c r="Q132" s="32" t="n">
-        <v>20.98</v>
+        <v>22.14</v>
       </c>
       <c r="R132" s="23" t="inlineStr">
         <is>
@@ -14298,13 +14308,13 @@
       </c>
       <c r="N133" s="2" t="n"/>
       <c r="O133" s="32" t="n">
-        <v>13.1</v>
+        <v>14.4</v>
       </c>
       <c r="P133" s="32" t="n">
-        <v>25.2</v>
+        <v>24.3</v>
       </c>
       <c r="Q133" s="32" t="n">
-        <v>19.39</v>
+        <v>19.05</v>
       </c>
       <c r="R133" s="23" t="inlineStr">
         <is>
@@ -14520,13 +14530,13 @@
       </c>
       <c r="N135" s="2" t="n"/>
       <c r="O135" s="32" t="n">
-        <v>16.2</v>
+        <v>19.1</v>
       </c>
       <c r="P135" s="32" t="n">
-        <v>24.2</v>
+        <v>28</v>
       </c>
       <c r="Q135" s="32" t="n">
-        <v>19.43</v>
+        <v>21.84</v>
       </c>
       <c r="R135" s="23" t="inlineStr">
         <is>
@@ -14636,13 +14646,13 @@
       </c>
       <c r="N136" s="2" t="n"/>
       <c r="O136" s="32" t="n">
-        <v>17.8</v>
+        <v>20.1</v>
       </c>
       <c r="P136" s="32" t="n">
-        <v>26.4</v>
+        <v>25.2</v>
       </c>
       <c r="Q136" s="32" t="n">
-        <v>21.48</v>
+        <v>22.07</v>
       </c>
       <c r="R136" s="23" t="inlineStr">
         <is>
@@ -14752,13 +14762,13 @@
       </c>
       <c r="N137" s="2" t="n"/>
       <c r="O137" s="32" t="n">
-        <v>14.7</v>
+        <v>20</v>
       </c>
       <c r="P137" s="32" t="n">
-        <v>25.8</v>
+        <v>25.6</v>
       </c>
       <c r="Q137" s="32" t="n">
-        <v>19.44</v>
+        <v>21.96</v>
       </c>
       <c r="R137" s="23" t="inlineStr">
         <is>
@@ -14868,13 +14878,13 @@
       </c>
       <c r="N138" s="2" t="n"/>
       <c r="O138" s="32" t="n">
-        <v>14.8</v>
+        <v>16.1</v>
       </c>
       <c r="P138" s="32" t="n">
-        <v>23</v>
+        <v>24.5</v>
       </c>
       <c r="Q138" s="32" t="n">
-        <v>17.89</v>
+        <v>19.74</v>
       </c>
       <c r="R138" s="23" t="inlineStr">
         <is>
@@ -14984,13 +14994,13 @@
       </c>
       <c r="N139" s="2" t="n"/>
       <c r="O139" s="32" t="n">
-        <v>15.2</v>
+        <v>17.4</v>
       </c>
       <c r="P139" s="32" t="n">
-        <v>23.3</v>
+        <v>26</v>
       </c>
       <c r="Q139" s="32" t="n">
-        <v>18.38</v>
+        <v>21.04</v>
       </c>
       <c r="R139" s="23" t="inlineStr">
         <is>
@@ -15100,13 +15110,13 @@
       </c>
       <c r="N140" s="2" t="n"/>
       <c r="O140" s="32" t="n">
-        <v>16.3</v>
+        <v>16.7</v>
       </c>
       <c r="P140" s="32" t="n">
-        <v>23.2</v>
+        <v>29.8</v>
       </c>
       <c r="Q140" s="32" t="n">
-        <v>19.48</v>
+        <v>22.77</v>
       </c>
       <c r="R140" s="23" t="inlineStr">
         <is>
@@ -15318,13 +15328,13 @@
       </c>
       <c r="N142" s="2" t="n"/>
       <c r="O142" s="32" t="n">
-        <v>21.1</v>
+        <v>19.9</v>
       </c>
       <c r="P142" s="32" t="n">
-        <v>27.7</v>
+        <v>30.2</v>
       </c>
       <c r="Q142" s="32" t="n">
-        <v>23.57</v>
+        <v>24.01</v>
       </c>
       <c r="R142" s="23" t="inlineStr">
         <is>
@@ -15434,13 +15444,13 @@
       </c>
       <c r="N143" s="2" t="n"/>
       <c r="O143" s="32" t="n">
-        <v>22</v>
+        <v>21.9</v>
       </c>
       <c r="P143" s="32" t="n">
-        <v>26.9</v>
+        <v>30.8</v>
       </c>
       <c r="Q143" s="32" t="n">
-        <v>24.38</v>
+        <v>25.94</v>
       </c>
       <c r="R143" s="23" t="inlineStr">
         <is>
@@ -15750,13 +15760,13 @@
       </c>
       <c r="N146" s="2" t="n"/>
       <c r="O146" s="32" t="n">
-        <v>26.6</v>
+        <v>25.8</v>
       </c>
       <c r="P146" s="32" t="n">
-        <v>32.1</v>
+        <v>31.8</v>
       </c>
       <c r="Q146" s="32" t="n">
-        <v>28.96</v>
+        <v>28.85</v>
       </c>
       <c r="R146" s="23" t="inlineStr">
         <is>
@@ -15858,13 +15868,13 @@
       </c>
       <c r="N147" s="2" t="n"/>
       <c r="O147" s="32" t="n">
-        <v>19.9</v>
+        <v>24.1</v>
       </c>
       <c r="P147" s="32" t="n">
-        <v>25.2</v>
+        <v>29.4</v>
       </c>
       <c r="Q147" s="32" t="n">
-        <v>22.27</v>
+        <v>26.02</v>
       </c>
       <c r="R147" s="23" t="inlineStr">
         <is>
@@ -15974,13 +15984,13 @@
       </c>
       <c r="N148" s="2" t="n"/>
       <c r="O148" s="32" t="n">
-        <v>20.2</v>
+        <v>21.4</v>
       </c>
       <c r="P148" s="32" t="n">
-        <v>28.4</v>
+        <v>33.7</v>
       </c>
       <c r="Q148" s="32" t="n">
-        <v>22.76</v>
+        <v>25.77</v>
       </c>
       <c r="R148" s="23" t="inlineStr">
         <is>
@@ -16086,13 +16096,13 @@
       </c>
       <c r="N149" s="2" t="n"/>
       <c r="O149" s="32" t="n">
-        <v>9</v>
+        <v>12.3</v>
       </c>
       <c r="P149" s="32" t="n">
-        <v>16.6</v>
+        <v>23</v>
       </c>
       <c r="Q149" s="32" t="n">
-        <v>11.96</v>
+        <v>17.41</v>
       </c>
       <c r="R149" s="23" t="inlineStr">
         <is>
@@ -16202,13 +16212,13 @@
       </c>
       <c r="N150" s="2" t="n"/>
       <c r="O150" s="32" t="n">
-        <v>11.9</v>
+        <v>15.3</v>
       </c>
       <c r="P150" s="32" t="n">
-        <v>14.2</v>
+        <v>21.9</v>
       </c>
       <c r="Q150" s="32" t="n">
-        <v>13.01</v>
+        <v>18.71</v>
       </c>
       <c r="R150" s="23" t="inlineStr">
         <is>
@@ -16318,13 +16328,13 @@
       </c>
       <c r="N151" s="2" t="n"/>
       <c r="O151" s="32" t="n">
-        <v>19.1</v>
+        <v>20.7</v>
       </c>
       <c r="P151" s="32" t="n">
-        <v>23.6</v>
+        <v>26.4</v>
       </c>
       <c r="Q151" s="32" t="n">
-        <v>21.15</v>
+        <v>22.93</v>
       </c>
       <c r="R151" s="23" t="inlineStr">
         <is>
@@ -16524,13 +16534,13 @@
       </c>
       <c r="N153" s="2" t="n"/>
       <c r="O153" s="32" t="n">
-        <v>14.8</v>
+        <v>17.9</v>
       </c>
       <c r="P153" s="32" t="n">
-        <v>22.4</v>
+        <v>28.3</v>
       </c>
       <c r="Q153" s="32" t="n">
-        <v>18.48</v>
+        <v>21.96</v>
       </c>
       <c r="R153" s="23" t="inlineStr">
         <is>
@@ -16644,13 +16654,13 @@
       </c>
       <c r="N154" s="2" t="n"/>
       <c r="O154" s="32" t="n">
-        <v>3.5</v>
+        <v>4.9</v>
       </c>
       <c r="P154" s="32" t="n">
-        <v>18</v>
+        <v>18.9</v>
       </c>
       <c r="Q154" s="32" t="n">
-        <v>10.61</v>
+        <v>11.59</v>
       </c>
       <c r="R154" s="23" t="inlineStr">
         <is>
@@ -16944,13 +16954,13 @@
       </c>
       <c r="N157" s="2" t="n"/>
       <c r="O157" s="32" t="n">
-        <v>16.6</v>
+        <v>17.4</v>
       </c>
       <c r="P157" s="32" t="n">
-        <v>22.5</v>
+        <v>30.4</v>
       </c>
       <c r="Q157" s="32" t="n">
-        <v>19.25</v>
+        <v>22.02</v>
       </c>
       <c r="R157" s="23" t="inlineStr">
         <is>
@@ -17334,13 +17344,13 @@
       </c>
       <c r="N161" s="2" t="n"/>
       <c r="O161" s="32" t="n">
-        <v>4.1</v>
+        <v>9</v>
       </c>
       <c r="P161" s="32" t="n">
-        <v>22.9</v>
+        <v>22</v>
       </c>
       <c r="Q161" s="32" t="n">
-        <v>12.61</v>
+        <v>16.26</v>
       </c>
       <c r="R161" s="23" t="inlineStr">
         <is>
@@ -17449,12 +17459,8 @@
           <t>⚡</t>
         </is>
       </c>
-      <c r="O162" s="32" t="n">
-        <v>-10</v>
-      </c>
-      <c r="P162" s="32" t="n">
-        <v>12.9</v>
-      </c>
+      <c r="O162" s="32" t="n"/>
+      <c r="P162" s="32" t="n"/>
       <c r="Q162" s="32" t="n"/>
       <c r="R162" s="23" t="inlineStr">
         <is>
@@ -17559,8 +17565,12 @@
         </is>
       </c>
       <c r="N163" s="2" t="n"/>
-      <c r="O163" s="32" t="n"/>
-      <c r="P163" s="32" t="n"/>
+      <c r="O163" s="32" t="n">
+        <v>-7.2</v>
+      </c>
+      <c r="P163" s="32" t="n">
+        <v>14.3</v>
+      </c>
       <c r="Q163" s="32" t="n"/>
       <c r="R163" s="23" t="inlineStr">
         <is>
@@ -18310,10 +18320,10 @@
         </is>
       </c>
       <c r="O170" s="32" t="n">
-        <v>-4.9</v>
+        <v>-3</v>
       </c>
       <c r="P170" s="32" t="n">
-        <v>11.3</v>
+        <v>11.8</v>
       </c>
       <c r="Q170" s="32" t="n"/>
       <c r="R170" s="23" t="inlineStr">
@@ -18420,10 +18430,10 @@
       </c>
       <c r="N171" s="2" t="n"/>
       <c r="O171" s="32" t="n">
-        <v>-0.2</v>
+        <v>1.4</v>
       </c>
       <c r="P171" s="32" t="n">
-        <v>7.3</v>
+        <v>5.6</v>
       </c>
       <c r="Q171" s="32" t="n"/>
       <c r="R171" s="23" t="inlineStr">
@@ -18636,10 +18646,10 @@
       </c>
       <c r="N173" s="2" t="n"/>
       <c r="O173" s="32" t="n">
-        <v>-4.2</v>
+        <v>-1.3</v>
       </c>
       <c r="P173" s="32" t="n">
-        <v>8.199999999999999</v>
+        <v>10</v>
       </c>
       <c r="Q173" s="32" t="n"/>
       <c r="R173" s="23" t="inlineStr">
@@ -18741,12 +18751,8 @@
         </is>
       </c>
       <c r="N174" s="2" t="n"/>
-      <c r="O174" s="32" t="n">
-        <v>-7.3</v>
-      </c>
-      <c r="P174" s="32" t="n">
-        <v>-1.3</v>
-      </c>
+      <c r="O174" s="32" t="n"/>
+      <c r="P174" s="32" t="n"/>
       <c r="Q174" s="32" t="n"/>
       <c r="R174" s="23" t="inlineStr">
         <is>
@@ -18962,13 +18968,13 @@
       </c>
       <c r="N176" s="2" t="n"/>
       <c r="O176" s="32" t="n">
-        <v>4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="P176" s="32" t="n">
-        <v>12.4</v>
+        <v>15.4</v>
       </c>
       <c r="Q176" s="32" t="n">
-        <v>6.71</v>
+        <v>11.85</v>
       </c>
       <c r="R176" s="23" t="inlineStr">
         <is>
@@ -19066,13 +19072,13 @@
       </c>
       <c r="N177" s="2" t="n"/>
       <c r="O177" s="32" t="n">
-        <v>-8.6</v>
+        <v>-5.9</v>
       </c>
       <c r="P177" s="32" t="n">
-        <v>-2.8</v>
+        <v>0.4</v>
       </c>
       <c r="Q177" s="32" t="n">
-        <v>-5.88</v>
+        <v>-2.65</v>
       </c>
       <c r="R177" s="23" t="inlineStr">
         <is>
@@ -22585,10 +22591,10 @@
       </c>
       <c r="N213" s="2" t="n"/>
       <c r="O213" s="32" t="n">
-        <v>-10.7</v>
+        <v>-11.2</v>
       </c>
       <c r="P213" s="32" t="n">
-        <v>13.1</v>
+        <v>13.3</v>
       </c>
       <c r="Q213" s="32" t="n"/>
       <c r="R213" s="23" t="inlineStr">
@@ -25243,10 +25249,10 @@
       </c>
       <c r="N240" s="2" t="n"/>
       <c r="O240" s="32" t="n">
-        <v>-8.800000000000001</v>
+        <v>-11.5</v>
       </c>
       <c r="P240" s="32" t="n">
-        <v>-3.5</v>
+        <v>-1.4</v>
       </c>
       <c r="Q240" s="32" t="n"/>
       <c r="R240" s="23" t="inlineStr">
@@ -27687,10 +27693,10 @@
       </c>
       <c r="N265" s="2" t="n"/>
       <c r="O265" s="32" t="n">
-        <v>-59.8</v>
+        <v>-67.59999999999999</v>
       </c>
       <c r="P265" s="32" t="n">
-        <v>-51.9</v>
+        <v>-66.5</v>
       </c>
       <c r="Q265" s="32" t="n"/>
       <c r="R265" s="23" t="inlineStr">
@@ -30527,10 +30533,10 @@
       </c>
       <c r="N295" s="2" t="n"/>
       <c r="O295" s="32" t="n">
-        <v>-10.9</v>
+        <v>-16.9</v>
       </c>
       <c r="P295" s="32" t="n">
-        <v>4.1</v>
+        <v>-5.6</v>
       </c>
       <c r="Q295" s="32" t="n"/>
       <c r="R295" s="23" t="inlineStr">
@@ -31120,15 +31126,9 @@
         </is>
       </c>
       <c r="N301" s="2" t="n"/>
-      <c r="O301" s="32" t="n">
-        <v>23.2</v>
-      </c>
-      <c r="P301" s="32" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="Q301" s="32" t="n">
-        <v>27.2</v>
-      </c>
+      <c r="O301" s="32" t="n"/>
+      <c r="P301" s="32" t="n"/>
+      <c r="Q301" s="32" t="n"/>
       <c r="R301" s="23" t="inlineStr">
         <is>
           <t>Y</t>
@@ -31518,15 +31518,9 @@
         </is>
       </c>
       <c r="N305" s="2" t="n"/>
-      <c r="O305" s="32" t="n">
-        <v>-12.5</v>
-      </c>
-      <c r="P305" s="32" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="Q305" s="32" t="n">
-        <v>-3.38</v>
-      </c>
+      <c r="O305" s="32" t="n"/>
+      <c r="P305" s="32" t="n"/>
+      <c r="Q305" s="32" t="n"/>
       <c r="R305" s="23" t="inlineStr">
         <is>
           <t>Y</t>
@@ -31834,12 +31828,8 @@
         </is>
       </c>
       <c r="N308" s="2" t="n"/>
-      <c r="O308" s="32" t="n">
-        <v>-16.1</v>
-      </c>
-      <c r="P308" s="32" t="n">
-        <v>-3.7</v>
-      </c>
+      <c r="O308" s="32" t="n"/>
+      <c r="P308" s="32" t="n"/>
       <c r="Q308" s="32" t="n"/>
       <c r="R308" s="23" t="inlineStr">
         <is>
@@ -32037,11 +32027,7 @@
       <c r="O310" s="32" t="n"/>
       <c r="P310" s="32" t="n"/>
       <c r="Q310" s="32" t="n"/>
-      <c r="R310" s="23" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="R310" s="23" t="n"/>
       <c r="S310" s="37" t="n"/>
       <c r="T310" s="41" t="inlineStr">
         <is>
@@ -32084,109 +32070,309 @@
       <c r="AH310" s="2" t="n"/>
     </row>
     <row r="311" ht="24" customHeight="1" s="50">
-      <c r="A311" s="2" t="n"/>
-      <c r="B311" s="2" t="n"/>
-      <c r="C311" s="46" t="n"/>
-      <c r="D311" s="2" t="n"/>
-      <c r="E311" s="4" t="n"/>
+      <c r="A311" s="2" t="n">
+        <v>310</v>
+      </c>
+      <c r="B311" s="2" t="inlineStr">
+        <is>
+          <t>rp5</t>
+        </is>
+      </c>
+      <c r="C311" s="46" t="inlineStr">
+        <is>
+          <t>47639</t>
+        </is>
+      </c>
+      <c r="D311" s="2" t="inlineStr">
+        <is>
+          <t>Fujisan</t>
+        </is>
+      </c>
+      <c r="E311" s="4" t="n">
+        <v>99999</v>
+      </c>
       <c r="F311" s="39" t="n"/>
-      <c r="G311" s="29" t="n"/>
-      <c r="H311" s="29" t="n"/>
-      <c r="I311" s="2" t="n"/>
-      <c r="J311" s="27" t="n"/>
-      <c r="K311" s="4" t="n"/>
+      <c r="G311" s="29" t="n">
+        <v>35.367</v>
+      </c>
+      <c r="H311" s="29" t="n">
+        <v>138.733</v>
+      </c>
+      <c r="I311" s="2" t="n">
+        <v>3777.5</v>
+      </c>
+      <c r="J311" s="27" t="n">
+        <v>12</v>
+      </c>
+      <c r="K311" s="31" t="inlineStr">
+        <is>
+          <t>🇯🇵</t>
+        </is>
+      </c>
       <c r="L311" s="2" t="n"/>
-      <c r="M311" s="14" t="n"/>
+      <c r="M311" s="17" t="inlineStr">
+        <is>
+          <t>富士山</t>
+        </is>
+      </c>
       <c r="N311" s="2" t="n"/>
-      <c r="O311" s="32" t="n"/>
-      <c r="P311" s="32" t="n"/>
-      <c r="Q311" s="32" t="n"/>
-      <c r="R311" s="23" t="n"/>
+      <c r="O311" s="32" t="n">
+        <v>-5.8</v>
+      </c>
+      <c r="P311" s="32" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q311" s="32" t="n">
+        <v>-1.82</v>
+      </c>
+      <c r="R311" s="23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="S311" s="37" t="n"/>
-      <c r="T311" s="41" t="n"/>
-      <c r="U311" s="2" t="n"/>
-      <c r="V311" s="4" t="n"/>
-      <c r="W311" s="4" t="n"/>
-      <c r="X311" s="4" t="n"/>
+      <c r="T311" s="41" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="U311" s="2" t="inlineStr">
+        <is>
+          <t>中部地方</t>
+        </is>
+      </c>
+      <c r="V311" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="W311" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="X311" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="Y311" s="4" t="n"/>
       <c r="Z311" s="2" t="n"/>
       <c r="AA311" s="2" t="n"/>
       <c r="AB311" s="2" t="n"/>
       <c r="AC311" s="2" t="n"/>
-      <c r="AD311" s="2" t="n"/>
-      <c r="AE311" s="4" t="n"/>
+      <c r="AD311" s="2" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="AE311" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="AF311" s="4" t="n"/>
       <c r="AG311" s="2" t="n"/>
       <c r="AH311" s="2" t="n"/>
     </row>
     <row r="312" ht="24" customHeight="1" s="50">
-      <c r="A312" s="2" t="n"/>
+      <c r="A312" s="2" t="n">
+        <v>311</v>
+      </c>
       <c r="B312" s="2" t="n"/>
-      <c r="C312" s="46" t="n"/>
+      <c r="C312" s="46" t="inlineStr">
+        <is>
+          <t>56673</t>
+        </is>
+      </c>
       <c r="D312" s="2" t="n"/>
-      <c r="E312" s="4" t="n"/>
+      <c r="E312" s="4" t="n">
+        <v>99999</v>
+      </c>
       <c r="F312" s="39" t="n"/>
-      <c r="G312" s="29" t="n"/>
-      <c r="H312" s="29" t="n"/>
-      <c r="I312" s="2" t="n"/>
-      <c r="J312" s="27" t="n"/>
-      <c r="K312" s="4" t="n"/>
+      <c r="G312" s="29" t="n">
+        <v>26.9181</v>
+      </c>
+      <c r="H312" s="29" t="n">
+        <v>102.9267</v>
+      </c>
+      <c r="I312" s="2" t="n">
+        <v>893.9</v>
+      </c>
+      <c r="J312" s="27" t="n">
+        <v>12</v>
+      </c>
+      <c r="K312" s="31" t="inlineStr">
+        <is>
+          <t>🇨🇳</t>
+        </is>
+      </c>
       <c r="L312" s="2" t="n"/>
-      <c r="M312" s="14" t="n"/>
+      <c r="M312" s="14" t="inlineStr">
+        <is>
+          <t>巧家</t>
+        </is>
+      </c>
       <c r="N312" s="2" t="n"/>
       <c r="O312" s="32" t="n"/>
       <c r="P312" s="32" t="n"/>
       <c r="Q312" s="32" t="n"/>
-      <c r="R312" s="23" t="n"/>
+      <c r="R312" s="23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="S312" s="37" t="n"/>
-      <c r="T312" s="41" t="n"/>
-      <c r="U312" s="2" t="n"/>
-      <c r="V312" s="4" t="n"/>
-      <c r="W312" s="4" t="n"/>
-      <c r="X312" s="4" t="n"/>
+      <c r="T312" s="41" t="inlineStr">
+        <is>
+          <t>云南</t>
+        </is>
+      </c>
+      <c r="U312" s="2" t="inlineStr">
+        <is>
+          <t>云南</t>
+        </is>
+      </c>
+      <c r="V312" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="W312" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="X312" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="Y312" s="4" t="n"/>
-      <c r="Z312" s="2" t="n"/>
-      <c r="AA312" s="2" t="n"/>
+      <c r="Z312" s="2" t="inlineStr">
+        <is>
+          <t>昭通市</t>
+        </is>
+      </c>
+      <c r="AA312" s="2" t="inlineStr">
+        <is>
+          <t>巧家县</t>
+        </is>
+      </c>
       <c r="AB312" s="2" t="n"/>
       <c r="AC312" s="2" t="n"/>
-      <c r="AD312" s="2" t="n"/>
-      <c r="AE312" s="4" t="n"/>
+      <c r="AD312" s="2" t="inlineStr">
+        <is>
+          <t>中国</t>
+        </is>
+      </c>
+      <c r="AE312" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="AF312" s="4" t="n"/>
       <c r="AG312" s="2" t="n"/>
       <c r="AH312" s="2" t="n"/>
     </row>
     <row r="313" ht="24" customHeight="1" s="50">
-      <c r="A313" s="2" t="n"/>
-      <c r="B313" s="2" t="n"/>
-      <c r="C313" s="46" t="n"/>
-      <c r="D313" s="2" t="n"/>
-      <c r="E313" s="4" t="n"/>
+      <c r="A313" s="2" t="n">
+        <v>312</v>
+      </c>
+      <c r="B313" s="2" t="inlineStr">
+        <is>
+          <t>ogimet</t>
+        </is>
+      </c>
+      <c r="C313" s="46" t="inlineStr">
+        <is>
+          <t>24076</t>
+        </is>
+      </c>
+      <c r="D313" s="2" t="inlineStr">
+        <is>
+          <t>Deputatsky</t>
+        </is>
+      </c>
+      <c r="E313" s="4" t="n">
+        <v>99999</v>
+      </c>
       <c r="F313" s="39" t="n"/>
-      <c r="G313" s="29" t="n"/>
-      <c r="H313" s="29" t="n"/>
-      <c r="I313" s="2" t="n"/>
-      <c r="J313" s="27" t="n"/>
-      <c r="K313" s="4" t="n"/>
+      <c r="G313" s="29" t="n">
+        <v>69.33</v>
+      </c>
+      <c r="H313" s="29" t="n">
+        <v>139.6697</v>
+      </c>
+      <c r="I313" s="2" t="n">
+        <v>282</v>
+      </c>
+      <c r="J313" s="27" t="n">
+        <v>15</v>
+      </c>
+      <c r="K313" s="31" t="inlineStr">
+        <is>
+          <t>🇷🇺</t>
+        </is>
+      </c>
       <c r="L313" s="2" t="n"/>
-      <c r="M313" s="14" t="n"/>
+      <c r="M313" s="16" t="inlineStr">
+        <is>
+          <t>Deputatskii</t>
+        </is>
+      </c>
       <c r="N313" s="2" t="n"/>
-      <c r="O313" s="32" t="n"/>
-      <c r="P313" s="32" t="n"/>
-      <c r="Q313" s="32" t="n"/>
-      <c r="R313" s="23" t="n"/>
+      <c r="O313" s="32" t="n">
+        <v>-24.2</v>
+      </c>
+      <c r="P313" s="32" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="Q313" s="32" t="n">
+        <v>-9.84</v>
+      </c>
+      <c r="R313" s="23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="S313" s="37" t="n"/>
-      <c r="T313" s="41" t="n"/>
-      <c r="U313" s="2" t="n"/>
-      <c r="V313" s="4" t="n"/>
+      <c r="T313" s="41" t="inlineStr">
+        <is>
+          <t>雅库特</t>
+        </is>
+      </c>
+      <c r="U313" s="2" t="inlineStr">
+        <is>
+          <t>萨哈共和国</t>
+        </is>
+      </c>
+      <c r="V313" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="W313" s="4" t="n"/>
-      <c r="X313" s="4" t="n"/>
+      <c r="X313" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="Y313" s="4" t="n"/>
       <c r="Z313" s="2" t="n"/>
       <c r="AA313" s="2" t="n"/>
       <c r="AB313" s="2" t="n"/>
       <c r="AC313" s="2" t="n"/>
-      <c r="AD313" s="2" t="n"/>
-      <c r="AE313" s="4" t="n"/>
+      <c r="AD313" s="2" t="inlineStr">
+        <is>
+          <t>俄罗斯</t>
+        </is>
+      </c>
+      <c r="AE313" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
       <c r="AF313" s="4" t="n"/>
       <c r="AG313" s="2" t="n"/>
       <c r="AH313" s="2" t="n"/>

</xml_diff>